<commit_message>
Versuch O11 fertig gemessen
</commit_message>
<xml_diff>
--- a/GP2/Versuch_O11/Messdaten_O11.xlsx
+++ b/GP2/Versuch_O11/Messdaten_O11.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fynnlucca/Documents/Grundpraktikum-1/GP2/Versuch_O11/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A353A5-FBA3-9144-B4E3-2A955930FC4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A6187D0-5064-4D4C-82D0-ED360B0806EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{C3015D50-456D-5A4E-B1A8-746D43650E4C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="23">
   <si>
     <t>Grundpraktikum</t>
   </si>
@@ -63,6 +63,48 @@
   </si>
   <si>
     <t>phi = 45°</t>
+  </si>
+  <si>
+    <t>Aufgabe 2</t>
+  </si>
+  <si>
+    <t>Blackbox 1</t>
+  </si>
+  <si>
+    <t>Ohne lamda/4 Plättchen</t>
+  </si>
+  <si>
+    <t>Minimum bei 7° mit Intensität 1.1894 V</t>
+  </si>
+  <si>
+    <t>Maximum zwischen -66 und -90 grad mit 1.6560 V</t>
+  </si>
+  <si>
+    <t>Nach einbringen des Lamda/4 Plättchen bei schnelle Achse 7°</t>
+  </si>
+  <si>
+    <t>Minimum bei -5° mit Intensität 1.0773</t>
+  </si>
+  <si>
+    <t>Blackbox 2</t>
+  </si>
+  <si>
+    <t>Messreihe</t>
+  </si>
+  <si>
+    <t>Ohne lambda/4</t>
+  </si>
+  <si>
+    <t>Mit lambda/4 Plättchen auf ca 7°</t>
+  </si>
+  <si>
+    <t>Lambda/4 Plättchen jetzt auf 8° da dort unser Maximum ist</t>
+  </si>
+  <si>
+    <t>Blackbox 3</t>
+  </si>
+  <si>
+    <t>Lambda/4 Plättchen am Minimum bei ca 33°</t>
   </si>
 </sst>
 </file>
@@ -434,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B366B8C-BB1B-9347-A52E-B8BEE5928BD5}">
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:AB74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
@@ -866,7 +908,842 @@
         <v>0.65359999999999996</v>
       </c>
     </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>14</v>
+      </c>
+      <c r="L46" t="s">
+        <v>16</v>
+      </c>
+      <c r="W46" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="L50" t="s">
+        <v>17</v>
+      </c>
+      <c r="W50" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="51" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="53" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>18</v>
+      </c>
+      <c r="E53" t="s">
+        <v>19</v>
+      </c>
+      <c r="L53" t="s">
+        <v>18</v>
+      </c>
+      <c r="P53" t="s">
+        <v>20</v>
+      </c>
+      <c r="W53" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA53" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="55" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>3</v>
+      </c>
+      <c r="B55" t="s">
+        <v>4</v>
+      </c>
+      <c r="E55" t="s">
+        <v>3</v>
+      </c>
+      <c r="F55" t="s">
+        <v>4</v>
+      </c>
+      <c r="L55" t="s">
+        <v>3</v>
+      </c>
+      <c r="M55" t="s">
+        <v>4</v>
+      </c>
+      <c r="P55" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>4</v>
+      </c>
+      <c r="W55" t="s">
+        <v>3</v>
+      </c>
+      <c r="X55" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA55" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB55" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>-90</v>
+      </c>
+      <c r="B56">
+        <v>1.6566000000000001</v>
+      </c>
+      <c r="E56">
+        <v>-90</v>
+      </c>
+      <c r="F56">
+        <v>1.4847999999999999</v>
+      </c>
+      <c r="L56">
+        <v>-90</v>
+      </c>
+      <c r="M56">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="P56">
+        <v>-90</v>
+      </c>
+      <c r="Q56">
+        <v>4.99E-2</v>
+      </c>
+      <c r="W56">
+        <v>-90</v>
+      </c>
+      <c r="X56">
+        <v>0.75090000000000001</v>
+      </c>
+      <c r="AA56">
+        <v>-90</v>
+      </c>
+      <c r="AB56">
+        <v>1.0790999999999999</v>
+      </c>
+    </row>
+    <row r="57" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>-80</v>
+      </c>
+      <c r="B57">
+        <v>1.6566000000000001</v>
+      </c>
+      <c r="E57">
+        <v>-80</v>
+      </c>
+      <c r="F57">
+        <v>1.4520999999999999</v>
+      </c>
+      <c r="L57">
+        <v>-80</v>
+      </c>
+      <c r="M57">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="P57">
+        <v>-80</v>
+      </c>
+      <c r="Q57">
+        <v>0.1016</v>
+      </c>
+      <c r="W57">
+        <v>-80</v>
+      </c>
+      <c r="X57">
+        <v>0.78949999999999998</v>
+      </c>
+      <c r="AA57">
+        <v>-80</v>
+      </c>
+      <c r="AB57">
+        <v>1.1448</v>
+      </c>
+    </row>
+    <row r="58" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>-70</v>
+      </c>
+      <c r="B58">
+        <v>1.6561999999999999</v>
+      </c>
+      <c r="E58">
+        <v>-70</v>
+      </c>
+      <c r="F58">
+        <v>1.3994</v>
+      </c>
+      <c r="L58">
+        <v>-70</v>
+      </c>
+      <c r="M58">
+        <v>4.5100000000000001E-2</v>
+      </c>
+      <c r="P58">
+        <v>-70</v>
+      </c>
+      <c r="Q58">
+        <v>0.17929999999999999</v>
+      </c>
+      <c r="W58">
+        <v>-70</v>
+      </c>
+      <c r="X58">
+        <v>0.81079999999999997</v>
+      </c>
+      <c r="AA58">
+        <v>-70</v>
+      </c>
+      <c r="AB58">
+        <v>1.1449</v>
+      </c>
+    </row>
+    <row r="59" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>-60</v>
+      </c>
+      <c r="B59">
+        <v>1.6007</v>
+      </c>
+      <c r="E59">
+        <v>-60</v>
+      </c>
+      <c r="F59">
+        <v>1.3251999999999999</v>
+      </c>
+      <c r="L59">
+        <v>-60</v>
+      </c>
+      <c r="M59">
+        <v>0.13550000000000001</v>
+      </c>
+      <c r="P59">
+        <v>-60</v>
+      </c>
+      <c r="Q59">
+        <v>0.28720000000000001</v>
+      </c>
+      <c r="W59">
+        <v>-60</v>
+      </c>
+      <c r="X59">
+        <v>0.81720000000000004</v>
+      </c>
+      <c r="AA59">
+        <v>-60</v>
+      </c>
+      <c r="AB59">
+        <v>1.0806</v>
+      </c>
+    </row>
+    <row r="60" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>-50</v>
+      </c>
+      <c r="B60">
+        <v>1.5224</v>
+      </c>
+      <c r="E60">
+        <v>-50</v>
+      </c>
+      <c r="F60">
+        <v>1.2567999999999999</v>
+      </c>
+      <c r="L60">
+        <v>-50</v>
+      </c>
+      <c r="M60">
+        <v>0.26329999999999998</v>
+      </c>
+      <c r="P60">
+        <v>-50</v>
+      </c>
+      <c r="Q60">
+        <v>0.40710000000000002</v>
+      </c>
+      <c r="W60">
+        <v>-50</v>
+      </c>
+      <c r="X60">
+        <v>0.81359999999999999</v>
+      </c>
+      <c r="AA60">
+        <v>-50</v>
+      </c>
+      <c r="AB60">
+        <v>0.95309999999999995</v>
+      </c>
+    </row>
+    <row r="61" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>-40</v>
+      </c>
+      <c r="B61">
+        <v>1.4244000000000001</v>
+      </c>
+      <c r="E61">
+        <v>-40</v>
+      </c>
+      <c r="F61">
+        <v>1.1855</v>
+      </c>
+      <c r="L61">
+        <v>-40</v>
+      </c>
+      <c r="M61">
+        <v>0.41520000000000001</v>
+      </c>
+      <c r="P61">
+        <v>-40</v>
+      </c>
+      <c r="Q61">
+        <v>0.51749999999999996</v>
+      </c>
+      <c r="W61">
+        <v>-40</v>
+      </c>
+      <c r="X61">
+        <v>0.78569999999999995</v>
+      </c>
+      <c r="AA61">
+        <v>-40</v>
+      </c>
+      <c r="AB61">
+        <v>0.7853</v>
+      </c>
+    </row>
+    <row r="62" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>-30</v>
+      </c>
+      <c r="B62">
+        <v>1.3479000000000001</v>
+      </c>
+      <c r="E62">
+        <v>-30</v>
+      </c>
+      <c r="F62">
+        <v>1.1231</v>
+      </c>
+      <c r="L62">
+        <v>-30</v>
+      </c>
+      <c r="M62">
+        <v>0.56299999999999994</v>
+      </c>
+      <c r="P62">
+        <v>-30</v>
+      </c>
+      <c r="Q62">
+        <v>0.61850000000000005</v>
+      </c>
+      <c r="W62">
+        <v>-30</v>
+      </c>
+      <c r="X62">
+        <v>0.74750000000000005</v>
+      </c>
+      <c r="AA62">
+        <v>-30</v>
+      </c>
+      <c r="AB62">
+        <v>0.5635</v>
+      </c>
+    </row>
+    <row r="63" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>-20</v>
+      </c>
+      <c r="B63">
+        <v>1.2685</v>
+      </c>
+      <c r="E63">
+        <v>-20</v>
+      </c>
+      <c r="F63">
+        <v>1.0859000000000001</v>
+      </c>
+      <c r="L63">
+        <v>-20</v>
+      </c>
+      <c r="M63">
+        <v>0.6925</v>
+      </c>
+      <c r="P63">
+        <v>-20</v>
+      </c>
+      <c r="Q63">
+        <v>0.69279999999999997</v>
+      </c>
+      <c r="W63">
+        <v>-20</v>
+      </c>
+      <c r="X63">
+        <v>0.70079999999999998</v>
+      </c>
+      <c r="AA63">
+        <v>-20</v>
+      </c>
+      <c r="AB63">
+        <v>0.37190000000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>-10</v>
+      </c>
+      <c r="B64">
+        <v>1.2071000000000001</v>
+      </c>
+      <c r="E64">
+        <v>-10</v>
+      </c>
+      <c r="F64">
+        <v>1.0702</v>
+      </c>
+      <c r="L64">
+        <v>-10</v>
+      </c>
+      <c r="M64">
+        <v>0.78569999999999995</v>
+      </c>
+      <c r="P64">
+        <v>-10</v>
+      </c>
+      <c r="Q64">
+        <v>0.72189999999999999</v>
+      </c>
+      <c r="W64">
+        <v>-10</v>
+      </c>
+      <c r="X64">
+        <v>0.65049999999999997</v>
+      </c>
+      <c r="AA64">
+        <v>-10</v>
+      </c>
+      <c r="AB64">
+        <v>0.20669999999999999</v>
+      </c>
+    </row>
+    <row r="65" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>0</v>
+      </c>
+      <c r="B65">
+        <v>1.1802999999999999</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>1.0706</v>
+      </c>
+      <c r="L65">
+        <v>0</v>
+      </c>
+      <c r="M65">
+        <v>0.8427</v>
+      </c>
+      <c r="P65">
+        <v>0</v>
+      </c>
+      <c r="Q65">
+        <v>0.72070000000000001</v>
+      </c>
+      <c r="W65">
+        <v>0</v>
+      </c>
+      <c r="X65">
+        <v>0.60440000000000005</v>
+      </c>
+      <c r="AA65">
+        <v>0</v>
+      </c>
+      <c r="AB65">
+        <v>7.3599999999999999E-2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>10</v>
+      </c>
+      <c r="B66">
+        <v>1.1791</v>
+      </c>
+      <c r="E66">
+        <v>10</v>
+      </c>
+      <c r="F66">
+        <v>1.1007</v>
+      </c>
+      <c r="L66">
+        <v>10</v>
+      </c>
+      <c r="M66">
+        <v>0.84730000000000005</v>
+      </c>
+      <c r="P66">
+        <v>10</v>
+      </c>
+      <c r="Q66">
+        <v>0.67110000000000003</v>
+      </c>
+      <c r="W66">
+        <v>10</v>
+      </c>
+      <c r="X66">
+        <v>0.56510000000000005</v>
+      </c>
+      <c r="AA66">
+        <v>10</v>
+      </c>
+      <c r="AB66">
+        <v>6.4999999999999997E-3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>20</v>
+      </c>
+      <c r="B67">
+        <v>1.2126999999999999</v>
+      </c>
+      <c r="E67">
+        <v>20</v>
+      </c>
+      <c r="F67">
+        <v>1.1536</v>
+      </c>
+      <c r="L67">
+        <v>20</v>
+      </c>
+      <c r="M67">
+        <v>0.79910000000000003</v>
+      </c>
+      <c r="P67">
+        <v>20</v>
+      </c>
+      <c r="Q67">
+        <v>0.58389999999999997</v>
+      </c>
+      <c r="W67">
+        <v>20</v>
+      </c>
+      <c r="X67">
+        <v>0.54049999999999998</v>
+      </c>
+      <c r="AA67">
+        <v>20</v>
+      </c>
+      <c r="AB67">
+        <v>6.1999999999999998E-3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>30</v>
+      </c>
+      <c r="B68">
+        <v>1.2710999999999999</v>
+      </c>
+      <c r="E68">
+        <v>30</v>
+      </c>
+      <c r="F68">
+        <v>1.2229000000000001</v>
+      </c>
+      <c r="L68">
+        <v>30</v>
+      </c>
+      <c r="M68">
+        <v>0.70940000000000003</v>
+      </c>
+      <c r="P68">
+        <v>30</v>
+      </c>
+      <c r="Q68">
+        <v>0.47720000000000001</v>
+      </c>
+      <c r="W68">
+        <v>30</v>
+      </c>
+      <c r="X68">
+        <v>0.53410000000000002</v>
+      </c>
+      <c r="AA68">
+        <v>30</v>
+      </c>
+      <c r="AB68">
+        <v>7.8799999999999995E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>40</v>
+      </c>
+      <c r="B69">
+        <v>1.3533999999999999</v>
+      </c>
+      <c r="E69">
+        <v>40</v>
+      </c>
+      <c r="F69">
+        <v>1.2926</v>
+      </c>
+      <c r="L69">
+        <v>40</v>
+      </c>
+      <c r="M69">
+        <v>0.57550000000000001</v>
+      </c>
+      <c r="P69">
+        <v>40</v>
+      </c>
+      <c r="Q69">
+        <v>0.35820000000000002</v>
+      </c>
+      <c r="W69">
+        <v>40</v>
+      </c>
+      <c r="X69">
+        <v>0.53939999999999999</v>
+      </c>
+      <c r="AA69">
+        <v>40</v>
+      </c>
+      <c r="AB69">
+        <v>0.21290000000000001</v>
+      </c>
+    </row>
+    <row r="70" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>50</v>
+      </c>
+      <c r="B70">
+        <v>1.4424999999999999</v>
+      </c>
+      <c r="E70">
+        <v>50</v>
+      </c>
+      <c r="F70">
+        <v>1.3656999999999999</v>
+      </c>
+      <c r="L70">
+        <v>50</v>
+      </c>
+      <c r="M70">
+        <v>0.438</v>
+      </c>
+      <c r="P70">
+        <v>50</v>
+      </c>
+      <c r="Q70">
+        <v>0.2445</v>
+      </c>
+      <c r="W70">
+        <v>50</v>
+      </c>
+      <c r="X70">
+        <v>0.56820000000000004</v>
+      </c>
+      <c r="AA70">
+        <v>50</v>
+      </c>
+      <c r="AB70">
+        <v>0.39069999999999999</v>
+      </c>
+    </row>
+    <row r="71" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>60</v>
+      </c>
+      <c r="B71">
+        <v>1.5356000000000001</v>
+      </c>
+      <c r="E71">
+        <v>60</v>
+      </c>
+      <c r="F71">
+        <v>1.4307000000000001</v>
+      </c>
+      <c r="L71">
+        <v>60</v>
+      </c>
+      <c r="M71">
+        <v>0.28639999999999999</v>
+      </c>
+      <c r="P71">
+        <v>60</v>
+      </c>
+      <c r="Q71">
+        <v>0.1404</v>
+      </c>
+      <c r="W71">
+        <v>60</v>
+      </c>
+      <c r="X71">
+        <v>0.60470000000000002</v>
+      </c>
+      <c r="AA71">
+        <v>60</v>
+      </c>
+      <c r="AB71">
+        <v>0.58020000000000005</v>
+      </c>
+    </row>
+    <row r="72" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>70</v>
+      </c>
+      <c r="B72">
+        <v>1.6109</v>
+      </c>
+      <c r="E72">
+        <v>70</v>
+      </c>
+      <c r="F72">
+        <v>1.4774</v>
+      </c>
+      <c r="L72">
+        <v>70</v>
+      </c>
+      <c r="M72">
+        <v>0.15110000000000001</v>
+      </c>
+      <c r="P72">
+        <v>70</v>
+      </c>
+      <c r="Q72">
+        <v>7.5800000000000006E-2</v>
+      </c>
+      <c r="W72">
+        <v>70</v>
+      </c>
+      <c r="X72">
+        <v>0.65249999999999997</v>
+      </c>
+      <c r="AA72">
+        <v>70</v>
+      </c>
+      <c r="AB72">
+        <v>0.77200000000000002</v>
+      </c>
+    </row>
+    <row r="73" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>80</v>
+      </c>
+      <c r="B73">
+        <v>1.6533</v>
+      </c>
+      <c r="E73">
+        <v>80</v>
+      </c>
+      <c r="F73">
+        <v>1.4959</v>
+      </c>
+      <c r="L73">
+        <v>80</v>
+      </c>
+      <c r="M73">
+        <v>5.6599999999999998E-2</v>
+      </c>
+      <c r="P73">
+        <v>80</v>
+      </c>
+      <c r="Q73">
+        <v>4.1099999999999998E-2</v>
+      </c>
+      <c r="W73">
+        <v>80</v>
+      </c>
+      <c r="X73">
+        <v>0.70350000000000001</v>
+      </c>
+      <c r="AA73">
+        <v>80</v>
+      </c>
+      <c r="AB73">
+        <v>0.9466</v>
+      </c>
+    </row>
+    <row r="74" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>90</v>
+      </c>
+      <c r="B74">
+        <v>1.655</v>
+      </c>
+      <c r="E74">
+        <v>90</v>
+      </c>
+      <c r="F74">
+        <v>1.4833000000000001</v>
+      </c>
+      <c r="L74">
+        <v>90</v>
+      </c>
+      <c r="M74">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="P74">
+        <v>90</v>
+      </c>
+      <c r="Q74">
+        <v>4.87E-2</v>
+      </c>
+      <c r="W74">
+        <v>90</v>
+      </c>
+      <c r="X74">
+        <v>0.74909999999999999</v>
+      </c>
+      <c r="AA74">
+        <v>90</v>
+      </c>
+      <c r="AB74">
+        <v>1.0710999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>